<commit_message>
Add the four いるかのせなか。product photos
These shots are portrait, not square like the つるりんちょ。ones, so size
each picture from its own dimensions and keep the aspect ratio rather
than forcing a square. Column H no longer reads なし for those rows.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013PR57qgwoN4kM429aZRbXL
</commit_message>
<xml_diff>
--- a/biteki-bestcosme/【髪にドラマを】美的2027年1月号・美的MEN「下半期ベストコスメ」リサーチアンケート.xlsx
+++ b/biteki-bestcosme/【髪にドラマを】美的2027年1月号・美的MEN「下半期ベストコスメ」リサーチアンケート.xlsx
@@ -2305,6 +2305,138 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>498842</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="897791" cy="1257300"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="いるかのせなか。オイル"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="897791" cy="1257300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>498842</xdr:colOff>
+      <xdr:row>68</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="897791" cy="1257300"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="19" name="いるかのせなか。CMCミルク"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="897791" cy="1257300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>498842</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="897791" cy="1257300"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="20" name="いるかのせなか。フォーム"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="897791" cy="1257300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>498842</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="897791" cy="1257300"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="21" name="いるかのせなか。ミスト"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="897791" cy="1257300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -3927,7 +4059,7 @@
       </c>
       <c r="K67" s="23"/>
     </row>
-    <row r="68" spans="1:11" ht="58.8" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:11" ht="105" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A68" s="46" t="s">
         <v>56</v>
       </c>
@@ -3957,11 +4089,7 @@
           <t xml:space="preserve">80mL</t>
         </is>
       </c>
-      <c r="H68" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">なし</t>
-        </is>
-      </c>
+      <c r="H68" s="43"/>
       <c r="I68" s="44">
         <v>46249</v>
       </c>
@@ -3970,7 +4098,7 @@
       </c>
       <c r="K68" s="23"/>
     </row>
-    <row r="69" spans="1:11" ht="58.8" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:11" ht="105" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A69" s="46" t="inlineStr">
         <is>
           <t xml:space="preserve">ライフスタイル</t>
@@ -4007,11 +4135,7 @@
           <t xml:space="preserve">140g</t>
         </is>
       </c>
-      <c r="H69" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">なし</t>
-        </is>
-      </c>
+      <c r="H69" s="43"/>
       <c r="I69" s="44">
         <v>46249</v>
       </c>
@@ -4020,7 +4144,7 @@
       </c>
       <c r="K69" s="23"/>
     </row>
-    <row r="70" spans="1:11" ht="58.8" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:11" ht="105" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A70" s="46" t="inlineStr">
         <is>
           <t xml:space="preserve">ライフスタイル</t>
@@ -4057,11 +4181,7 @@
           <t xml:space="preserve">180mL</t>
         </is>
       </c>
-      <c r="H70" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">なし</t>
-        </is>
-      </c>
+      <c r="H70" s="43"/>
       <c r="I70" s="44">
         <v>46249</v>
       </c>
@@ -4070,7 +4190,7 @@
       </c>
       <c r="K70" s="23"/>
     </row>
-    <row r="71" spans="1:11" ht="58.8" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:11" ht="105" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A71" s="46" t="inlineStr">
         <is>
           <t xml:space="preserve">ライフスタイル</t>
@@ -4107,11 +4227,7 @@
           <t xml:space="preserve">150mL</t>
         </is>
       </c>
-      <c r="H71" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">なし</t>
-        </is>
-      </c>
+      <c r="H71" s="43"/>
       <c r="I71" s="44">
         <v>46249</v>
       </c>

</xml_diff>